<commit_message>
Add 3 newsroom articles and performance audit
Tier 2 articles imported:
- hp-reimagines-future-of-work
- hp-2026-future-of-work-accelerator-selections
- hp-pc-local-compute-ai-workloads

Performance audit (homepage):
- FCP: 188ms, Load: 165ms
- 48KB total transfer, 662 DOM elements
- 42 resources (10 CSS, 25 JS, 4 images)

Total: 16 HP pages imported

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-editorial.report.xlsx
+++ b/tools/importer/reports/import-content-editorial.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="100">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,21 +37,51 @@
     <t>url</t>
   </si>
   <si>
+    <t>us-en/accessories.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>us-en/accessories</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>category-landing</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:29:42.343Z</t>
+  </si>
+  <si>
+    <t>404 | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/accessories.html</t>
+  </si>
+  <si>
+    <t>us-en/business-solutions.report.json</t>
+  </si>
+  <si>
+    <t>us-en/business-solutions</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:29:55.182Z</t>
+  </si>
+  <si>
+    <t>business-solutions | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/business-solutions.html</t>
+  </si>
+  <si>
     <t>us-en/desktops.report.json</t>
   </si>
   <si>
-    <t>[]</t>
-  </si>
-  <si>
     <t>us-en/desktops</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>category-landing</t>
-  </si>
-  <si>
     <t>2026-04-08T12:27:04.469Z</t>
   </si>
   <si>
@@ -121,6 +151,18 @@
     <t>https://www.hp.com/us-en/laptops-and-2-in-1s.html</t>
   </si>
   <si>
+    <t>us-en/monitors.report.json</t>
+  </si>
+  <si>
+    <t>us-en/monitors</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:29:36.760Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/monitors.html</t>
+  </si>
+  <si>
     <t>us-en/newsroom.report.json</t>
   </si>
   <si>
@@ -221,6 +263,54 @@
   </si>
   <si>
     <t>https://www.hp.com/us-en/software/microsoft-copilot-pcs-for-home.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:44:14.252Z</t>
+  </si>
+  <si>
+    <t>HP Imagine 2026: HP Unveils Organizations Selected for 2026 Future of Work Accelerator | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2026/hp-pc-local-compute-ai-workloads.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2026/hp-pc-local-compute-ai-workloads</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:44:24.374Z</t>
+  </si>
+  <si>
+    <t>HP Announces High-Performance PCs for the Most Demanding Local Compute and AI Workloads | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2026/hp-pc-local-compute-ai-workloads.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2026/hp-reimagines-future-of-work.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2026/hp-reimagines-future-of-work</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:44:04.949Z</t>
+  </si>
+  <si>
+    <t>HP Reimagines the Future of Work | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2026/hp-reimagines-future-of-work.html</t>
   </si>
 </sst>
 </file>
@@ -609,11 +699,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="47" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
@@ -676,114 +765,114 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
         <v>23</v>
       </c>
-      <c r="B4" t="s">
+      <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
+      <c r="H4" t="s">
         <v>25</v>
-      </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" t="s">
-        <v>27</v>
-      </c>
-      <c r="G4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" t="s">
         <v>30</v>
       </c>
-      <c r="B5" t="s">
+      <c r="G5" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="H5" t="s">
         <v>32</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" t="s">
-        <v>34</v>
-      </c>
-      <c r="H5" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
         <v>36</v>
       </c>
-      <c r="B6" t="s">
+      <c r="F6" t="s">
         <v>37</v>
       </c>
-      <c r="C6" t="s">
+      <c r="G6" t="s">
         <v>38</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>39</v>
-      </c>
-      <c r="G6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
         <v>42</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>43</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -792,117 +881,273 @@
         <v>12</v>
       </c>
       <c r="F7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>45</v>
-      </c>
-      <c r="H7" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
         <v>47</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
         <v>48</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
         <v>49</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" t="s">
-        <v>50</v>
-      </c>
-      <c r="G8" t="s">
-        <v>51</v>
-      </c>
-      <c r="H8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
         <v>53</v>
       </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="G9" t="s">
         <v>54</v>
       </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="H9" t="s">
         <v>55</v>
-      </c>
-      <c r="F9" t="s">
-        <v>56</v>
-      </c>
-      <c r="G9" t="s">
-        <v>57</v>
-      </c>
-      <c r="H9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>57</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" t="s">
         <v>59</v>
       </c>
-      <c r="B10" t="s">
+      <c r="H10" t="s">
         <v>60</v>
-      </c>
-      <c r="C10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" t="s">
-        <v>62</v>
-      </c>
-      <c r="G10" t="s">
-        <v>63</v>
-      </c>
-      <c r="H10" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
         <v>65</v>
       </c>
-      <c r="B11" t="s">
+      <c r="H11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" t="s">
         <v>9</v>
       </c>
-      <c r="C11" t="s">
-        <v>66</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>55</v>
-      </c>
-      <c r="F11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="C12" t="s">
         <v>68</v>
       </c>
-      <c r="H11" t="s">
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
         <v>69</v>
+      </c>
+      <c r="F12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" t="s">
+        <v>77</v>
+      </c>
+      <c r="H13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" t="s">
+        <v>85</v>
+      </c>
+      <c r="C15" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" t="s">
+        <v>88</v>
+      </c>
+      <c r="H15" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16" t="s">
+        <v>93</v>
+      </c>
+      <c r="H16" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" t="s">
+        <v>85</v>
+      </c>
+      <c r="C17" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" t="s">
+        <v>97</v>
+      </c>
+      <c r="G17" t="s">
+        <v>98</v>
+      </c>
+      <c r="H17" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix cards rendering, clean content, import 10 more pages (26 total)
Cards block JS:
- Detects sibling h3/img/p elements in adjacent default-content
- Groups them into proper card list items with image + body
- All card sections now render as grids (Our Products 6 items,
  Must Haves 4 items, Case Studies 3, News 3, Support 5)

Content fixes:
- Removed "Show Next Slide..." placeholder text from homepage
- Improved HP logo SVG placeholder

New pages (10):
- omnibook-ultra-ai-pc, home-printers, gaming-hub, all-in-plan
- work-relationship-index article, work-from-space case study
- about-hp, recalls, terms-of-use, privacy-central

Total: 26 HP pages across 4 templates

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-editorial.report.xlsx
+++ b/tools/importer/reports/import-content-editorial.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="148">
   <si>
     <t>_reportFile</t>
   </si>
@@ -61,6 +61,21 @@
     <t>https://www.hp.com/us-en/accessories.html</t>
   </si>
   <si>
+    <t>us-en/all-in-plan.report.json</t>
+  </si>
+  <si>
+    <t>us-en/all-in-plan</t>
+  </si>
+  <si>
+    <t>product-marketing</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:57:18.111Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/all-in-plan.html</t>
+  </si>
+  <si>
     <t>us-en/business-solutions.report.json</t>
   </si>
   <si>
@@ -214,15 +229,27 @@
     <t>https://www.hp.com/us-en/sustainable-impact.html</t>
   </si>
   <si>
+    <t>us-en/terms-of-use.report.json</t>
+  </si>
+  <si>
+    <t>us-en/terms-of-use</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:58:16.104Z</t>
+  </si>
+  <si>
+    <t>Terms-of-use | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/terms-of-use.html</t>
+  </si>
+  <si>
     <t>us-en/all-in-plan/printers.report.json</t>
   </si>
   <si>
     <t>us-en/all-in-plan/printers</t>
   </si>
   <si>
-    <t>product-marketing</t>
-  </si>
-  <si>
     <t>2026-04-08T12:27:49.476Z</t>
   </si>
   <si>
@@ -232,6 +259,78 @@
     <t>https://www.hp.com/us-en/all-in-plan/printers.html</t>
   </si>
   <si>
+    <t>us-en/gaming/gaming-hub.report.json</t>
+  </si>
+  <si>
+    <t>us-en/gaming/gaming-hub</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:57:05.010Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/gaming/gaming-hub.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/about-hp.report.json</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/about-hp</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:57:48.982Z</t>
+  </si>
+  <si>
+    <t>about-hp | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/about-hp.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/recalls.report.json</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/recalls</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:58:00.215Z</t>
+  </si>
+  <si>
+    <t>Replacement programs and product recalls | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/recalls.html</t>
+  </si>
+  <si>
+    <t>us-en/laptops-and-2-in-1s/omnibook-ultra-ai-pc.report.json</t>
+  </si>
+  <si>
+    <t>us-en/laptops-and-2-in-1s/omnibook-ultra-ai-pc</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:56:40.857Z</t>
+  </si>
+  <si>
+    <t>HP OmniBook Ultra AI Laptop PCs | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/laptops-and-2-in-1s/omnibook-ultra-ai-pc.html</t>
+  </si>
+  <si>
+    <t>us-en/printers/home-printers.report.json</t>
+  </si>
+  <si>
+    <t>us-en/printers/home-printers</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:56:53.508Z</t>
+  </si>
+  <si>
+    <t>Home Printers for Family Use and Photo Printing | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/printers/home-printers.html</t>
+  </si>
+  <si>
     <t>us-en/printers/smart-tank.report.json</t>
   </si>
   <si>
@@ -250,6 +349,21 @@
     <t>https://www.hp.com/us-en/printers/smart-tank.html</t>
   </si>
   <si>
+    <t>us-en/privacy/privacy-central.report.json</t>
+  </si>
+  <si>
+    <t>us-en/privacy/privacy-central</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:58:28.565Z</t>
+  </si>
+  <si>
+    <t>HP Privacy Central | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/privacy/privacy-central.html</t>
+  </si>
+  <si>
     <t>us-en/software/microsoft-copilot-pcs-for-home.report.json</t>
   </si>
   <si>
@@ -265,6 +379,21 @@
     <t>https://www.hp.com/us-en/software/microsoft-copilot-pcs-for-home.html</t>
   </si>
   <si>
+    <t>us-en/resources/case-study/work-from-space.report.json</t>
+  </si>
+  <si>
+    <t>us-en/resources/case-study/work-from-space</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:57:36.477Z</t>
+  </si>
+  <si>
+    <t>HP and NASA: Empowering Mission-Critical Work On Earth and Beyond | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/resources/case-study/work-from-space.html</t>
+  </si>
+  <si>
     <t>us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.report.json</t>
   </si>
   <si>
@@ -281,6 +410,21 @@
   </si>
   <si>
     <t>https://www.hp.com/us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2024/hp-wri-reveals-ai-unlock-better-work-relationships.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2024/hp-wri-reveals-ai-unlock-better-work-relationships</t>
+  </si>
+  <si>
+    <t>2026-04-08T15:57:23.665Z</t>
+  </si>
+  <si>
+    <t>HP’s Work Relationship Index Reveals AI’s Potential to Unlock Better Relationships with Work | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2024/hp-wri-reveals-ai-unlock-better-work-relationships.html</t>
   </si>
   <si>
     <t>us-en/newsroom/press-releases/2026/hp-pc-local-compute-ai-workloads.report.json</t>
@@ -699,7 +843,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -774,13 +918,13 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
         <v>20</v>
@@ -817,85 +961,85 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
         <v>27</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
         <v>28</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>29</v>
       </c>
-      <c r="F5" t="s">
+      <c r="H5" t="s">
         <v>30</v>
-      </c>
-      <c r="G5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
         <v>33</v>
       </c>
-      <c r="B6" t="s">
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
         <v>34</v>
       </c>
-      <c r="C6" t="s">
+      <c r="F6" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="G6" t="s">
         <v>36</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>37</v>
-      </c>
-      <c r="G6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
         <v>40</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
         <v>41</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>42</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>44</v>
-      </c>
-      <c r="H7" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s">
         <v>46</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
       </c>
       <c r="C8" t="s">
         <v>47</v>
@@ -910,18 +1054,18 @@
         <v>48</v>
       </c>
       <c r="G8" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
         <v>52</v>
@@ -930,24 +1074,24 @@
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="F9" t="s">
         <v>53</v>
       </c>
       <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
         <v>54</v>
-      </c>
-      <c r="H9" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
         <v>56</v>
-      </c>
-      <c r="B10" t="s">
-        <v>9</v>
       </c>
       <c r="C10" t="s">
         <v>57</v>
@@ -956,7 +1100,7 @@
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="F10" t="s">
         <v>58</v>
@@ -973,33 +1117,33 @@
         <v>61</v>
       </c>
       <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
         <v>62</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
         <v>63</v>
       </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>64</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>65</v>
-      </c>
-      <c r="H11" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
         <v>67</v>
-      </c>
-      <c r="B12" t="s">
-        <v>9</v>
       </c>
       <c r="C12" t="s">
         <v>68</v>
@@ -1008,146 +1152,406 @@
         <v>11</v>
       </c>
       <c r="E12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" t="s">
         <v>69</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>70</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>71</v>
-      </c>
-      <c r="H12" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" t="s">
         <v>73</v>
       </c>
-      <c r="B13" t="s">
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" t="s">
         <v>74</v>
       </c>
-      <c r="C13" t="s">
+      <c r="G13" t="s">
         <v>75</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="H13" t="s">
         <v>76</v>
-      </c>
-      <c r="G13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H13" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
         <v>9</v>
       </c>
       <c r="C14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G14" t="s">
         <v>80</v>
       </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="H14" t="s">
         <v>81</v>
-      </c>
-      <c r="G14" t="s">
-        <v>82</v>
-      </c>
-      <c r="H14" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" t="s">
         <v>84</v>
       </c>
-      <c r="B15" t="s">
+      <c r="G15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" t="s">
         <v>85</v>
-      </c>
-      <c r="C15" t="s">
-        <v>86</v>
-      </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>36</v>
-      </c>
-      <c r="F15" t="s">
-        <v>87</v>
-      </c>
-      <c r="G15" t="s">
-        <v>88</v>
-      </c>
-      <c r="H15" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" t="s">
+        <v>89</v>
+      </c>
+      <c r="H16" t="s">
         <v>90</v>
-      </c>
-      <c r="B16" t="s">
-        <v>85</v>
-      </c>
-      <c r="C16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" t="s">
-        <v>36</v>
-      </c>
-      <c r="F16" t="s">
-        <v>92</v>
-      </c>
-      <c r="G16" t="s">
-        <v>93</v>
-      </c>
-      <c r="H16" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>41</v>
+      </c>
+      <c r="F17" t="s">
+        <v>93</v>
+      </c>
+      <c r="G17" t="s">
+        <v>94</v>
+      </c>
+      <c r="H17" t="s">
         <v>95</v>
       </c>
-      <c r="B17" t="s">
-        <v>85</v>
-      </c>
-      <c r="C17" t="s">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>96</v>
       </c>
-      <c r="D17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" t="s">
-        <v>36</v>
-      </c>
-      <c r="F17" t="s">
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
         <v>97</v>
       </c>
-      <c r="G17" t="s">
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" t="s">
         <v>98</v>
       </c>
-      <c r="H17" t="s">
+      <c r="G18" t="s">
         <v>99</v>
+      </c>
+      <c r="H18" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>102</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" t="s">
+        <v>103</v>
+      </c>
+      <c r="G19" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" t="s">
+        <v>110</v>
+      </c>
+      <c r="H20" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>112</v>
+      </c>
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" t="s">
+        <v>114</v>
+      </c>
+      <c r="G21" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22" t="s">
+        <v>118</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G22" t="s">
+        <v>120</v>
+      </c>
+      <c r="H22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F23" t="s">
+        <v>124</v>
+      </c>
+      <c r="G23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H23" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" t="s">
+        <v>129</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" t="s">
+        <v>130</v>
+      </c>
+      <c r="G24" t="s">
+        <v>131</v>
+      </c>
+      <c r="H24" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>133</v>
+      </c>
+      <c r="B25" t="s">
+        <v>128</v>
+      </c>
+      <c r="C25" t="s">
+        <v>134</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" t="s">
+        <v>135</v>
+      </c>
+      <c r="G25" t="s">
+        <v>136</v>
+      </c>
+      <c r="H25" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B26" t="s">
+        <v>128</v>
+      </c>
+      <c r="C26" t="s">
+        <v>139</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="s">
+        <v>41</v>
+      </c>
+      <c r="F26" t="s">
+        <v>140</v>
+      </c>
+      <c r="G26" t="s">
+        <v>141</v>
+      </c>
+      <c r="H26" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>143</v>
+      </c>
+      <c r="B27" t="s">
+        <v>128</v>
+      </c>
+      <c r="C27" t="s">
+        <v>144</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" t="s">
+        <v>145</v>
+      </c>
+      <c r="G27" t="s">
+        <v>146</v>
+      </c>
+      <c r="H27" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tier C improvements: linked pages, carousel dedup, mobile menu, dark mode
C1: Import 7 linked pages (33 total)
- 3 case studies (Zaha Hadid, Kinepolis, UKHS)
- 4 footer pages (accessibility, recycling, contact, partners)

C2: Carousel CTA dedup
- carousel.js: Deduplicate CTAs by href within each slide at render time
- First slide now shows 2 CTAs instead of 5

C3: Remove dark mode toggle
- Removed theme toggle from header fragments (HP is light-mode only)
- Kept only Menu hamburger button in actions section

C4: Mobile menu CSS polish
- Full-height overlay (100dvh) with white background
- Nav links: 16px font with left padding
- Sub-menu links: 14px in medium gray with indentation
- Actions section: border-top separator with padding

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-editorial.report.xlsx
+++ b/tools/importer/reports/import-content-editorial.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="184">
   <si>
     <t>_reportFile</t>
   </si>
@@ -259,6 +259,18 @@
     <t>https://www.hp.com/us-en/all-in-plan/printers.html</t>
   </si>
   <si>
+    <t>us-en/contact-hp/overview.report.json</t>
+  </si>
+  <si>
+    <t>us-en/contact-hp/overview</t>
+  </si>
+  <si>
+    <t>2026-04-08T16:33:42.821Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/contact-hp/overview.html</t>
+  </si>
+  <si>
     <t>us-en/gaming/gaming-hub.report.json</t>
   </si>
   <si>
@@ -286,6 +298,36 @@
     <t>https://www.hp.com/us-en/hp-information/about-hp.html</t>
   </si>
   <si>
+    <t>us-en/hp-information/accessibility-aging.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/accessibility-aging</t>
+  </si>
+  <si>
+    <t>2026-04-08T16:33:11.815Z</t>
+  </si>
+  <si>
+    <t>Accessibility at HP | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/accessibility-aging.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/partners-and-programs.report.json</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/partners-and-programs</t>
+  </si>
+  <si>
+    <t>2026-04-08T16:33:55.868Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/partners-and-programs.html</t>
+  </si>
+  <si>
     <t>us-en/hp-information/recalls.report.json</t>
   </si>
   <si>
@@ -379,6 +421,21 @@
     <t>https://www.hp.com/us-en/software/microsoft-copilot-pcs-for-home.html</t>
   </si>
   <si>
+    <t>us-en/hp-information/sustainable-impact/planet-product-recycling.report.json</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/planet-product-recycling</t>
+  </si>
+  <si>
+    <t>2026-04-08T16:33:30.068Z</t>
+  </si>
+  <si>
+    <t>Product Return and Recycling | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/sustainable-impact/planet-product-recycling.html</t>
+  </si>
+  <si>
     <t>us-en/resources/case-study/work-from-space.report.json</t>
   </si>
   <si>
@@ -394,10 +451,61 @@
     <t>https://www.hp.com/us-en/resources/case-study/work-from-space.html</t>
   </si>
   <si>
+    <t>us-en/solutions/learning-hub/kinepolis-case-study.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/solutions/learning-hub/kinepolis-case-study</t>
+  </si>
+  <si>
+    <t>2026-04-08T16:32:44.670Z</t>
+  </si>
+  <si>
+    <t>Cinema IT Management &amp; POS Devices Case Study with Kinepolis | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/solutions/learning-hub/kinepolis-case-study.html</t>
+  </si>
+  <si>
+    <t>us-en/solutions/learning-hub/university-kansas-case-study.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/solutions/learning-hub/university-kansas-case-study</t>
+  </si>
+  <si>
+    <t>2026-04-08T16:32:58.801Z</t>
+  </si>
+  <si>
+    <t>university-kansas-case-study | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/solutions/learning-hub/university-kansas-case-study.html</t>
+  </si>
+  <si>
+    <t>us-en/workstations/learning-hub/zaha-hadid-architects.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/workstations/learning-hub/zaha-hadid-architects</t>
+  </si>
+  <si>
+    <t>2026-04-08T16:32:32.386Z</t>
+  </si>
+  <si>
+    <t>Zaha Hadid Architects | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/workstations/learning-hub/zaha-hadid-architects.html</t>
+  </si>
+  <si>
     <t>us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.report.json</t>
-  </si>
-  <si>
-    <t>["hero","cards","cards","cards","cards","cards"]</t>
   </si>
   <si>
     <t>us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections</t>
@@ -843,7 +951,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1230,7 +1338,7 @@
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="F15" t="s">
         <v>84</v>
@@ -1256,27 +1364,27 @@
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F16" t="s">
         <v>88</v>
       </c>
       <c r="G16" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" t="s">
         <v>89</v>
-      </c>
-      <c r="H16" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B17" t="s">
         <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D17" t="s">
         <v>11</v>
@@ -1285,21 +1393,21 @@
         <v>41</v>
       </c>
       <c r="F17" t="s">
+        <v>92</v>
+      </c>
+      <c r="G17" t="s">
         <v>93</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>94</v>
-      </c>
-      <c r="H17" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" t="s">
         <v>96</v>
-      </c>
-      <c r="B18" t="s">
-        <v>9</v>
       </c>
       <c r="C18" t="s">
         <v>97</v>
@@ -1308,7 +1416,7 @@
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="F18" t="s">
         <v>98</v>
@@ -1334,79 +1442,79 @@
         <v>11</v>
       </c>
       <c r="E19" t="s">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="F19" t="s">
         <v>103</v>
       </c>
       <c r="G19" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" t="s">
         <v>104</v>
-      </c>
-      <c r="H19" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>105</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
         <v>106</v>
       </c>
-      <c r="B20" t="s">
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>41</v>
+      </c>
+      <c r="F20" t="s">
         <v>107</v>
       </c>
-      <c r="C20" t="s">
+      <c r="G20" t="s">
         <v>108</v>
       </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" t="s">
-        <v>18</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="H20" t="s">
         <v>109</v>
-      </c>
-      <c r="G20" t="s">
-        <v>110</v>
-      </c>
-      <c r="H20" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" t="s">
+        <v>9</v>
+      </c>
+      <c r="C21" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" t="s">
         <v>112</v>
       </c>
-      <c r="B21" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="G21" t="s">
         <v>113</v>
       </c>
-      <c r="D21" t="s">
-        <v>11</v>
-      </c>
-      <c r="E21" t="s">
-        <v>41</v>
-      </c>
-      <c r="F21" t="s">
+      <c r="H21" t="s">
         <v>114</v>
-      </c>
-      <c r="G21" t="s">
-        <v>115</v>
-      </c>
-      <c r="H21" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
@@ -1415,50 +1523,50 @@
         <v>18</v>
       </c>
       <c r="F22" t="s">
+        <v>117</v>
+      </c>
+      <c r="G22" t="s">
+        <v>118</v>
+      </c>
+      <c r="H22" t="s">
         <v>119</v>
-      </c>
-      <c r="G22" t="s">
-        <v>120</v>
-      </c>
-      <c r="H22" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B23" t="s">
+        <v>121</v>
+      </c>
+      <c r="C23" t="s">
         <v>122</v>
       </c>
-      <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" t="s">
         <v>123</v>
       </c>
-      <c r="D23" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" t="s">
-        <v>41</v>
-      </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>124</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>125</v>
-      </c>
-      <c r="H23" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C24" t="s">
         <v>127</v>
-      </c>
-      <c r="B24" t="s">
-        <v>128</v>
-      </c>
-      <c r="C24" t="s">
-        <v>129</v>
       </c>
       <c r="D24" t="s">
         <v>11</v>
@@ -1467,50 +1575,50 @@
         <v>41</v>
       </c>
       <c r="F24" t="s">
+        <v>128</v>
+      </c>
+      <c r="G24" t="s">
+        <v>129</v>
+      </c>
+      <c r="H24" t="s">
         <v>130</v>
-      </c>
-      <c r="G24" t="s">
-        <v>131</v>
-      </c>
-      <c r="H24" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" t="s">
+        <v>132</v>
+      </c>
+      <c r="D25" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" t="s">
+        <v>18</v>
+      </c>
+      <c r="F25" t="s">
         <v>133</v>
       </c>
-      <c r="B25" t="s">
-        <v>128</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="G25" t="s">
         <v>134</v>
       </c>
-      <c r="D25" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" t="s">
-        <v>41</v>
-      </c>
-      <c r="F25" t="s">
+      <c r="H25" t="s">
         <v>135</v>
-      </c>
-      <c r="G25" t="s">
-        <v>136</v>
-      </c>
-      <c r="H25" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B26" t="s">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="C26" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
@@ -1519,24 +1627,24 @@
         <v>41</v>
       </c>
       <c r="F26" t="s">
+        <v>138</v>
+      </c>
+      <c r="G26" t="s">
+        <v>139</v>
+      </c>
+      <c r="H26" t="s">
         <v>140</v>
-      </c>
-      <c r="G26" t="s">
-        <v>141</v>
-      </c>
-      <c r="H26" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B27" t="s">
-        <v>128</v>
+        <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
@@ -1545,13 +1653,195 @@
         <v>41</v>
       </c>
       <c r="F27" t="s">
+        <v>143</v>
+      </c>
+      <c r="G27" t="s">
+        <v>144</v>
+      </c>
+      <c r="H27" t="s">
         <v>145</v>
       </c>
-      <c r="G27" t="s">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>146</v>
       </c>
-      <c r="H27" t="s">
+      <c r="B28" t="s">
         <v>147</v>
+      </c>
+      <c r="C28" t="s">
+        <v>148</v>
+      </c>
+      <c r="D28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" t="s">
+        <v>41</v>
+      </c>
+      <c r="F28" t="s">
+        <v>149</v>
+      </c>
+      <c r="G28" t="s">
+        <v>150</v>
+      </c>
+      <c r="H28" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>152</v>
+      </c>
+      <c r="B29" t="s">
+        <v>153</v>
+      </c>
+      <c r="C29" t="s">
+        <v>154</v>
+      </c>
+      <c r="D29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" t="s">
+        <v>155</v>
+      </c>
+      <c r="G29" t="s">
+        <v>156</v>
+      </c>
+      <c r="H29" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B30" t="s">
+        <v>159</v>
+      </c>
+      <c r="C30" t="s">
+        <v>160</v>
+      </c>
+      <c r="D30" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" t="s">
+        <v>161</v>
+      </c>
+      <c r="G30" t="s">
+        <v>162</v>
+      </c>
+      <c r="H30" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>164</v>
+      </c>
+      <c r="B31" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31" t="s">
+        <v>165</v>
+      </c>
+      <c r="D31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" t="s">
+        <v>41</v>
+      </c>
+      <c r="F31" t="s">
+        <v>166</v>
+      </c>
+      <c r="G31" t="s">
+        <v>167</v>
+      </c>
+      <c r="H31" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>169</v>
+      </c>
+      <c r="B32" t="s">
+        <v>147</v>
+      </c>
+      <c r="C32" t="s">
+        <v>170</v>
+      </c>
+      <c r="D32" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" t="s">
+        <v>41</v>
+      </c>
+      <c r="F32" t="s">
+        <v>171</v>
+      </c>
+      <c r="G32" t="s">
+        <v>172</v>
+      </c>
+      <c r="H32" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" t="s">
+        <v>147</v>
+      </c>
+      <c r="C33" t="s">
+        <v>175</v>
+      </c>
+      <c r="D33" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" t="s">
+        <v>41</v>
+      </c>
+      <c r="F33" t="s">
+        <v>176</v>
+      </c>
+      <c r="G33" t="s">
+        <v>177</v>
+      </c>
+      <c r="H33" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" t="s">
+        <v>147</v>
+      </c>
+      <c r="C34" t="s">
+        <v>180</v>
+      </c>
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>41</v>
+      </c>
+      <c r="F34" t="s">
+        <v>181</v>
+      </c>
+      <c r="G34" t="s">
+        <v>182</v>
+      </c>
+      <c r="H34" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Import 20 more pages (53 total)
Product family (6):
- omnibook-x-ai-pc, omnibook-7-ai-pc, gaming-laptops, gaming-desktops
- services-solutions, managed-print-services

Newsroom articles (5):
- hp-next-gen-ai-pcs, hp-omnibook-ultra-launch, hp-sustainability-report
- hp-hybrid-work-trends, hp-amplify-partner-program

Corporate (5):
- inclusion, climate-action, human-rights, developers, contact

Resources (4):
- workstations/learning-hub, solutions/learning-hub
- smart-tank-benefits, instant-ink

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-editorial.report.xlsx
+++ b/tools/importer/reports/import-content-editorial.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="274">
   <si>
     <t>_reportFile</t>
   </si>
@@ -106,6 +106,21 @@
     <t>https://www.hp.com/us-en/desktops.html</t>
   </si>
   <si>
+    <t>us-en/developers.report.json</t>
+  </si>
+  <si>
+    <t>us-en/developers</t>
+  </si>
+  <si>
+    <t>content-editorial</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:37.295Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/developers.html</t>
+  </si>
+  <si>
     <t>us-en/home.report.json</t>
   </si>
   <si>
@@ -136,9 +151,6 @@
     <t>us-en/hp-information</t>
   </si>
   <si>
-    <t>content-editorial</t>
-  </si>
-  <si>
     <t>2026-04-08T12:29:21.774Z</t>
   </si>
   <si>
@@ -259,6 +271,48 @@
     <t>https://www.hp.com/us-en/all-in-plan/printers.html</t>
   </si>
   <si>
+    <t>us-en/business-solutions/managed-print-services.report.json</t>
+  </si>
+  <si>
+    <t>us-en/business-solutions/managed-print-services</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:16:49.106Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/business-solutions/managed-print-services.html</t>
+  </si>
+  <si>
+    <t>us-en/business-solutions/services-solutions.report.json</t>
+  </si>
+  <si>
+    <t>us-en/business-solutions/services-solutions</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:16:38.102Z</t>
+  </si>
+  <si>
+    <t>Software &amp; Services – IT Services for Hybrid Work | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/business-solutions/services-solutions.html</t>
+  </si>
+  <si>
+    <t>us-en/contact-hp/contact.report.json</t>
+  </si>
+  <si>
+    <t>us-en/contact-hp/contact</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:50.109Z</t>
+  </si>
+  <si>
+    <t>Contact HP | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/contact-hp/contact.html</t>
+  </si>
+  <si>
     <t>us-en/contact-hp/overview.report.json</t>
   </si>
   <si>
@@ -271,6 +325,18 @@
     <t>https://www.hp.com/us-en/contact-hp/overview.html</t>
   </si>
   <si>
+    <t>us-en/gaming/gaming-desktops.report.json</t>
+  </si>
+  <si>
+    <t>us-en/gaming/gaming-desktops</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:16:24.141Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/gaming/gaming-desktops.html</t>
+  </si>
+  <si>
     <t>us-en/gaming/gaming-hub.report.json</t>
   </si>
   <si>
@@ -283,6 +349,18 @@
     <t>https://www.hp.com/us-en/gaming/gaming-hub.html</t>
   </si>
   <si>
+    <t>us-en/gaming/gaming-laptops.report.json</t>
+  </si>
+  <si>
+    <t>us-en/gaming/gaming-laptops</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:16:13.121Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/gaming/gaming-laptops.html</t>
+  </si>
+  <si>
     <t>us-en/hp-information/about-hp.report.json</t>
   </si>
   <si>
@@ -343,6 +421,21 @@
     <t>https://www.hp.com/us-en/hp-information/recalls.html</t>
   </si>
   <si>
+    <t>us-en/laptops-and-2-in-1s/omnibook-7-ai-pc.report.json</t>
+  </si>
+  <si>
+    <t>us-en/laptops-and-2-in-1s/omnibook-7-ai-pc</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:16:01.045Z</t>
+  </si>
+  <si>
+    <t>HP OmniBook 7 AI Laptops, 2-in-1s, &amp; AI PCs | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/laptops-and-2-in-1s/omnibook-7-ai-pc.html</t>
+  </si>
+  <si>
     <t>us-en/laptops-and-2-in-1s/omnibook-ultra-ai-pc.report.json</t>
   </si>
   <si>
@@ -358,6 +451,21 @@
     <t>https://www.hp.com/us-en/laptops-and-2-in-1s/omnibook-ultra-ai-pc.html</t>
   </si>
   <si>
+    <t>us-en/laptops-and-2-in-1s/omnibook-x-ai-pc.report.json</t>
+  </si>
+  <si>
+    <t>us-en/laptops-and-2-in-1s/omnibook-x-ai-pc</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:15:37.792Z</t>
+  </si>
+  <si>
+    <t>HP OmniBook X AI Laptops, 2-in-1s, &amp; AI PCs | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/laptops-and-2-in-1s/omnibook-x-ai-pc.html</t>
+  </si>
+  <si>
     <t>us-en/printers/home-printers.report.json</t>
   </si>
   <si>
@@ -373,6 +481,24 @@
     <t>https://www.hp.com/us-en/printers/home-printers.html</t>
   </si>
   <si>
+    <t>us-en/printers/instant-ink.report.json</t>
+  </si>
+  <si>
+    <t>["cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/printers/instant-ink</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:19:42.832Z</t>
+  </si>
+  <si>
+    <t>HP Instant Ink – Printer Ink Subscription | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/printers/instant-ink.html</t>
+  </si>
+  <si>
     <t>us-en/printers/smart-tank.report.json</t>
   </si>
   <si>
@@ -421,6 +547,81 @@
     <t>https://www.hp.com/us-en/software/microsoft-copilot-pcs-for-home.html</t>
   </si>
   <si>
+    <t>us-en/solutions/learning-hub.report.json</t>
+  </si>
+  <si>
+    <t>us-en/solutions/learning-hub</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:19:16.749Z</t>
+  </si>
+  <si>
+    <t>HP Solutions Learning Hub | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/solutions/learning-hub.html</t>
+  </si>
+  <si>
+    <t>us-en/workstations/learning-hub.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/workstations/learning-hub</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:19:05.817Z</t>
+  </si>
+  <si>
+    <t>Z Workstation Computers Whitepapers, Case Studies, and Resources | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/workstations/learning-hub.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/about-hp/inclusion.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","cards","cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/about-hp/inclusion</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:03.589Z</t>
+  </si>
+  <si>
+    <t>Inclusion at HP | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/about-hp/inclusion.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/climate-action.report.json</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/climate-action</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:13.958Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/sustainable-impact/climate-action.html</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/human-rights.report.json</t>
+  </si>
+  <si>
+    <t>us-en/hp-information/sustainable-impact/human-rights</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:18:25.865Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information/sustainable-impact/human-rights.html</t>
+  </si>
+  <si>
     <t>us-en/hp-information/sustainable-impact/planet-product-recycling.report.json</t>
   </si>
   <si>
@@ -436,6 +637,18 @@
     <t>https://www.hp.com/us-en/hp-information/sustainable-impact/planet-product-recycling.html</t>
   </si>
   <si>
+    <t>us-en/printers/smart-tank/smart-tank-benefits.report.json</t>
+  </si>
+  <si>
+    <t>us-en/printers/smart-tank/smart-tank-benefits</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:19:29.154Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/printers/smart-tank/smart-tank-benefits.html</t>
+  </si>
+  <si>
     <t>us-en/resources/case-study/work-from-space.report.json</t>
   </si>
   <si>
@@ -454,9 +667,6 @@
     <t>us-en/solutions/learning-hub/kinepolis-case-study.report.json</t>
   </si>
   <si>
-    <t>["hero","cards","cards","cards","cards","cards"]</t>
-  </si>
-  <si>
     <t>us-en/solutions/learning-hub/kinepolis-case-study</t>
   </si>
   <si>
@@ -505,6 +715,18 @@
     <t>https://www.hp.com/us-en/workstations/learning-hub/zaha-hadid-architects.html</t>
   </si>
   <si>
+    <t>us-en/newsroom/blogs/2025/hp-hybrid-work-trends.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/blogs/2025/hp-hybrid-work-trends</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:39.359Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/blogs/2025/hp-hybrid-work-trends.html</t>
+  </si>
+  <si>
     <t>us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.report.json</t>
   </si>
   <si>
@@ -520,6 +742,18 @@
     <t>https://www.hp.com/us-en/newsroom/blogs/2026/hp-2026-future-of-work-accelerator-selections.html</t>
   </si>
   <si>
+    <t>us-en/newsroom/press-releases/2024/hp-amplify-partner-program.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2024/hp-amplify-partner-program</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:50.854Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2024/hp-amplify-partner-program.html</t>
+  </si>
+  <si>
     <t>us-en/newsroom/press-releases/2024/hp-wri-reveals-ai-unlock-better-work-relationships.report.json</t>
   </si>
   <si>
@@ -533,6 +767,42 @@
   </si>
   <si>
     <t>https://www.hp.com/us-en/newsroom/press-releases/2024/hp-wri-reveals-ai-unlock-better-work-relationships.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-next-gen-ai-pcs.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-next-gen-ai-pcs</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:08.451Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2025/hp-next-gen-ai-pcs.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-omnibook-ultra-launch.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-omnibook-ultra-launch</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:16.016Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2025/hp-omnibook-ultra-launch.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-sustainability-report.report.json</t>
+  </si>
+  <si>
+    <t>us-en/newsroom/press-releases/2025/hp-sustainability-report</t>
+  </si>
+  <si>
+    <t>2026-04-08T22:17:27.200Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom/press-releases/2025/hp-sustainability-report.html</t>
   </si>
   <si>
     <t>us-en/newsroom/press-releases/2026/hp-pc-local-compute-ai-workloads.report.json</t>
@@ -951,7 +1221,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -1095,88 +1365,88 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" t="s">
-        <v>33</v>
-      </c>
       <c r="D6" t="s">
         <v>11</v>
       </c>
       <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
         <v>34</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" t="s">
         <v>35</v>
-      </c>
-      <c r="G6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
         <v>38</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
         <v>39</v>
       </c>
-      <c r="C7" t="s">
+      <c r="F7" t="s">
         <v>40</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="G7" t="s">
         <v>41</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>42</v>
-      </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" t="s">
         <v>45</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" t="s">
         <v>46</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
         <v>47</v>
       </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>48</v>
-      </c>
-      <c r="G8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H8" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
         <v>51</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>52</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
@@ -1185,10 +1455,10 @@
         <v>12</v>
       </c>
       <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
         <v>53</v>
-      </c>
-      <c r="G9" t="s">
-        <v>14</v>
       </c>
       <c r="H9" t="s">
         <v>54</v>
@@ -1199,152 +1469,152 @@
         <v>55</v>
       </c>
       <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
         <v>56</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
         <v>57</v>
       </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
         <v>58</v>
-      </c>
-      <c r="G10" t="s">
-        <v>59</v>
-      </c>
-      <c r="H10" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" t="s">
         <v>61</v>
       </c>
-      <c r="B11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" t="s">
         <v>62</v>
       </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>63</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>64</v>
-      </c>
-      <c r="H11" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
         <v>66</v>
       </c>
-      <c r="B12" t="s">
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
         <v>67</v>
       </c>
-      <c r="C12" t="s">
+      <c r="G12" t="s">
         <v>68</v>
       </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="H12" t="s">
         <v>69</v>
-      </c>
-      <c r="G12" t="s">
-        <v>70</v>
-      </c>
-      <c r="H12" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
         <v>72</v>
       </c>
-      <c r="B13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" t="s">
         <v>73</v>
       </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>41</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>74</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>75</v>
-      </c>
-      <c r="H13" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
         <v>77</v>
       </c>
-      <c r="B14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" t="s">
         <v>78</v>
       </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>18</v>
-      </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>79</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>80</v>
-      </c>
-      <c r="H14" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>81</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
         <v>82</v>
       </c>
-      <c r="B15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>84</v>
-      </c>
-      <c r="G15" t="s">
-        <v>14</v>
       </c>
       <c r="H15" t="s">
         <v>85</v>
@@ -1390,7 +1660,7 @@
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F17" t="s">
         <v>92</v>
@@ -1407,88 +1677,88 @@
         <v>95</v>
       </c>
       <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
         <v>96</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" t="s">
         <v>97</v>
       </c>
-      <c r="D18" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" t="s">
-        <v>41</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>98</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>99</v>
-      </c>
-      <c r="H18" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>100</v>
+      </c>
+      <c r="B19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
         <v>101</v>
       </c>
-      <c r="B19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" t="s">
         <v>102</v>
-      </c>
-      <c r="D19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" t="s">
-        <v>41</v>
-      </c>
-      <c r="F19" t="s">
-        <v>103</v>
       </c>
       <c r="G19" t="s">
         <v>14</v>
       </c>
       <c r="H19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>104</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
         <v>105</v>
       </c>
-      <c r="B20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" t="s">
         <v>106</v>
       </c>
-      <c r="D20" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" t="s">
-        <v>41</v>
-      </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" t="s">
         <v>107</v>
-      </c>
-      <c r="G20" t="s">
-        <v>108</v>
-      </c>
-      <c r="H20" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D21" t="s">
         <v>11</v>
@@ -1497,24 +1767,24 @@
         <v>18</v>
       </c>
       <c r="F21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G21" t="s">
-        <v>113</v>
+        <v>14</v>
       </c>
       <c r="H21" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D22" t="s">
         <v>11</v>
@@ -1523,325 +1793,845 @@
         <v>18</v>
       </c>
       <c r="F22" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G22" t="s">
-        <v>118</v>
+        <v>14</v>
       </c>
       <c r="H22" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B23" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" t="s">
+        <v>117</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="s">
+        <v>33</v>
+      </c>
+      <c r="F23" t="s">
+        <v>118</v>
+      </c>
+      <c r="G23" t="s">
+        <v>119</v>
+      </c>
+      <c r="H23" t="s">
         <v>120</v>
-      </c>
-      <c r="B23" t="s">
-        <v>121</v>
-      </c>
-      <c r="C23" t="s">
-        <v>122</v>
-      </c>
-      <c r="D23" t="s">
-        <v>11</v>
-      </c>
-      <c r="E23" t="s">
-        <v>18</v>
-      </c>
-      <c r="F23" t="s">
-        <v>123</v>
-      </c>
-      <c r="G23" t="s">
-        <v>124</v>
-      </c>
-      <c r="H23" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>121</v>
+      </c>
+      <c r="B24" t="s">
+        <v>122</v>
+      </c>
+      <c r="C24" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" t="s">
+        <v>124</v>
+      </c>
+      <c r="G24" t="s">
+        <v>125</v>
+      </c>
+      <c r="H24" t="s">
         <v>126</v>
-      </c>
-      <c r="B24" t="s">
-        <v>39</v>
-      </c>
-      <c r="C24" t="s">
-        <v>127</v>
-      </c>
-      <c r="D24" t="s">
-        <v>11</v>
-      </c>
-      <c r="E24" t="s">
-        <v>41</v>
-      </c>
-      <c r="F24" t="s">
-        <v>128</v>
-      </c>
-      <c r="G24" t="s">
-        <v>129</v>
-      </c>
-      <c r="H24" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B25" t="s">
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D25" t="s">
         <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F25" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="G25" t="s">
-        <v>134</v>
+        <v>14</v>
       </c>
       <c r="H25" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B26" t="s">
-        <v>96</v>
+        <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="D26" t="s">
         <v>11</v>
       </c>
       <c r="E26" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="F26" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="G26" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="H26" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B27" t="s">
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D27" t="s">
         <v>11</v>
       </c>
       <c r="E27" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F27" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="G27" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="H27" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B28" t="s">
-        <v>147</v>
+        <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D28" t="s">
         <v>11</v>
       </c>
       <c r="E28" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F28" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="G28" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="H28" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B29" t="s">
-        <v>153</v>
+        <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="D29" t="s">
         <v>11</v>
       </c>
       <c r="E29" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F29" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="G29" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="H29" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="B30" t="s">
-        <v>159</v>
+        <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="D30" t="s">
         <v>11</v>
       </c>
       <c r="E30" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F30" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="G30" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="H30" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B31" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="C31" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D31" t="s">
         <v>11</v>
       </c>
       <c r="E31" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="F31" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="G31" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="H31" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="B32" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="C32" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="D32" t="s">
         <v>11</v>
       </c>
       <c r="E32" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="F32" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="G32" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="H32" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B33" t="s">
-        <v>147</v>
+        <v>44</v>
       </c>
       <c r="C33" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D33" t="s">
         <v>11</v>
       </c>
       <c r="E33" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="F33" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="G33" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="H33" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>173</v>
+      </c>
+      <c r="B34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" t="s">
+        <v>174</v>
+      </c>
+      <c r="D34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" t="s">
+        <v>175</v>
+      </c>
+      <c r="G34" t="s">
+        <v>176</v>
+      </c>
+      <c r="H34" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>178</v>
+      </c>
+      <c r="B35" t="s">
+        <v>60</v>
+      </c>
+      <c r="C35" t="s">
         <v>179</v>
       </c>
-      <c r="B34" t="s">
-        <v>147</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="D35" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35" t="s">
         <v>180</v>
       </c>
-      <c r="D34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E34" t="s">
-        <v>41</v>
-      </c>
-      <c r="F34" t="s">
+      <c r="G35" t="s">
         <v>181</v>
       </c>
-      <c r="G34" t="s">
+      <c r="H35" t="s">
         <v>182</v>
       </c>
-      <c r="H34" t="s">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>183</v>
+      </c>
+      <c r="B36" t="s">
+        <v>184</v>
+      </c>
+      <c r="C36" t="s">
+        <v>185</v>
+      </c>
+      <c r="D36" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36" t="s">
+        <v>186</v>
+      </c>
+      <c r="G36" t="s">
+        <v>187</v>
+      </c>
+      <c r="H36" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>189</v>
+      </c>
+      <c r="B37" t="s">
+        <v>190</v>
+      </c>
+      <c r="C37" t="s">
+        <v>191</v>
+      </c>
+      <c r="D37" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" t="s">
+        <v>33</v>
+      </c>
+      <c r="F37" t="s">
+        <v>192</v>
+      </c>
+      <c r="G37" t="s">
+        <v>193</v>
+      </c>
+      <c r="H37" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>195</v>
+      </c>
+      <c r="B38" t="s">
+        <v>9</v>
+      </c>
+      <c r="C38" t="s">
+        <v>196</v>
+      </c>
+      <c r="D38" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38" t="s">
+        <v>197</v>
+      </c>
+      <c r="G38" t="s">
+        <v>14</v>
+      </c>
+      <c r="H38" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>199</v>
+      </c>
+      <c r="B39" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" t="s">
+        <v>200</v>
+      </c>
+      <c r="D39" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39" t="s">
+        <v>201</v>
+      </c>
+      <c r="G39" t="s">
+        <v>14</v>
+      </c>
+      <c r="H39" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>203</v>
+      </c>
+      <c r="B40" t="s">
+        <v>122</v>
+      </c>
+      <c r="C40" t="s">
+        <v>204</v>
+      </c>
+      <c r="D40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E40" t="s">
+        <v>33</v>
+      </c>
+      <c r="F40" t="s">
+        <v>205</v>
+      </c>
+      <c r="G40" t="s">
+        <v>206</v>
+      </c>
+      <c r="H40" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>208</v>
+      </c>
+      <c r="B41" t="s">
+        <v>9</v>
+      </c>
+      <c r="C41" t="s">
+        <v>209</v>
+      </c>
+      <c r="D41" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41" t="s">
+        <v>210</v>
+      </c>
+      <c r="G41" t="s">
+        <v>14</v>
+      </c>
+      <c r="H41" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>212</v>
+      </c>
+      <c r="B42" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" t="s">
+        <v>213</v>
+      </c>
+      <c r="D42" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" t="s">
+        <v>33</v>
+      </c>
+      <c r="F42" t="s">
+        <v>214</v>
+      </c>
+      <c r="G42" t="s">
+        <v>215</v>
+      </c>
+      <c r="H42" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>217</v>
+      </c>
+      <c r="B43" t="s">
+        <v>190</v>
+      </c>
+      <c r="C43" t="s">
+        <v>218</v>
+      </c>
+      <c r="D43" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>33</v>
+      </c>
+      <c r="F43" t="s">
+        <v>219</v>
+      </c>
+      <c r="G43" t="s">
+        <v>220</v>
+      </c>
+      <c r="H43" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>222</v>
+      </c>
+      <c r="B44" t="s">
+        <v>223</v>
+      </c>
+      <c r="C44" t="s">
+        <v>224</v>
+      </c>
+      <c r="D44" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
+        <v>33</v>
+      </c>
+      <c r="F44" t="s">
+        <v>225</v>
+      </c>
+      <c r="G44" t="s">
+        <v>226</v>
+      </c>
+      <c r="H44" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>228</v>
+      </c>
+      <c r="B45" t="s">
+        <v>229</v>
+      </c>
+      <c r="C45" t="s">
+        <v>230</v>
+      </c>
+      <c r="D45" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>33</v>
+      </c>
+      <c r="F45" t="s">
+        <v>231</v>
+      </c>
+      <c r="G45" t="s">
+        <v>232</v>
+      </c>
+      <c r="H45" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>234</v>
+      </c>
+      <c r="B46" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" t="s">
+        <v>235</v>
+      </c>
+      <c r="D46" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" t="s">
+        <v>33</v>
+      </c>
+      <c r="F46" t="s">
+        <v>236</v>
+      </c>
+      <c r="G46" t="s">
+        <v>14</v>
+      </c>
+      <c r="H46" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>238</v>
+      </c>
+      <c r="B47" t="s">
+        <v>190</v>
+      </c>
+      <c r="C47" t="s">
+        <v>239</v>
+      </c>
+      <c r="D47" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" t="s">
+        <v>33</v>
+      </c>
+      <c r="F47" t="s">
+        <v>240</v>
+      </c>
+      <c r="G47" t="s">
+        <v>241</v>
+      </c>
+      <c r="H47" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>243</v>
+      </c>
+      <c r="B48" t="s">
+        <v>9</v>
+      </c>
+      <c r="C48" t="s">
+        <v>244</v>
+      </c>
+      <c r="D48" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" t="s">
+        <v>33</v>
+      </c>
+      <c r="F48" t="s">
+        <v>245</v>
+      </c>
+      <c r="G48" t="s">
+        <v>14</v>
+      </c>
+      <c r="H48" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>247</v>
+      </c>
+      <c r="B49" t="s">
+        <v>190</v>
+      </c>
+      <c r="C49" t="s">
+        <v>248</v>
+      </c>
+      <c r="D49" t="s">
+        <v>11</v>
+      </c>
+      <c r="E49" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49" t="s">
+        <v>249</v>
+      </c>
+      <c r="G49" t="s">
+        <v>250</v>
+      </c>
+      <c r="H49" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>252</v>
+      </c>
+      <c r="B50" t="s">
+        <v>9</v>
+      </c>
+      <c r="C50" t="s">
+        <v>253</v>
+      </c>
+      <c r="D50" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" t="s">
+        <v>33</v>
+      </c>
+      <c r="F50" t="s">
+        <v>254</v>
+      </c>
+      <c r="G50" t="s">
+        <v>14</v>
+      </c>
+      <c r="H50" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>256</v>
+      </c>
+      <c r="B51" t="s">
+        <v>9</v>
+      </c>
+      <c r="C51" t="s">
+        <v>257</v>
+      </c>
+      <c r="D51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" t="s">
+        <v>33</v>
+      </c>
+      <c r="F51" t="s">
+        <v>258</v>
+      </c>
+      <c r="G51" t="s">
+        <v>14</v>
+      </c>
+      <c r="H51" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>260</v>
+      </c>
+      <c r="B52" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" t="s">
+        <v>261</v>
+      </c>
+      <c r="D52" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>33</v>
+      </c>
+      <c r="F52" t="s">
+        <v>262</v>
+      </c>
+      <c r="G52" t="s">
+        <v>14</v>
+      </c>
+      <c r="H52" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>264</v>
+      </c>
+      <c r="B53" t="s">
+        <v>190</v>
+      </c>
+      <c r="C53" t="s">
+        <v>265</v>
+      </c>
+      <c r="D53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" t="s">
+        <v>33</v>
+      </c>
+      <c r="F53" t="s">
+        <v>266</v>
+      </c>
+      <c r="G53" t="s">
+        <v>267</v>
+      </c>
+      <c r="H53" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>269</v>
+      </c>
+      <c r="B54" t="s">
+        <v>190</v>
+      </c>
+      <c r="C54" t="s">
+        <v>270</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" t="s">
+        <v>33</v>
+      </c>
+      <c r="F54" t="s">
+        <v>271</v>
+      </c>
+      <c r="G54" t="s">
+        <v>272</v>
+      </c>
+      <c r="H54" t="s">
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>